<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.002-03 Le pain doré de Sarah
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.002-03.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.002-03.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>hall, rue, vitrine de la boulangerie</t>
+          <t>hall au clou des clés, rue, vitrine de la boulangerie</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sarah veut voir le pain doré derrière la vitrine. Les clés tintent. Une manche du manteau jaune est tordue. Papa l'aide. Ils voient le pigeon et le pain. Le foulard et le manteau rentrent à leur place.</t>
+          <t>Un filet d'air passe sous la porte du hall. Il sent le pain de la rue. Sur le clou, un éclat de clé brille. Sarah veut le pain doré de la vitrine, maintenant. Elle tire le manteau jaune : la manche est à l'envers. Elle refuse de foncer, ouvre la manche, sort. Un cageot bloque la vitrine ; l'éclat de clé montre un trou. Sur la croûte, l'éclat de clé brille. Le manteau rentre au crochet.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Les clés de papa pendent à un clou. Elles font une petite chanson. Un foulard dort sur la rampe. Il est rayé, bleu et blanc. Sous la porte, un filet d'air froid. La rue sent déjà le pain. Sarah, tu as entendu les clés ? Oui, papa. Elles tintent. En ce moment, Sarah écoute les clés. Son manteau jaune attend au crochet. Le tissu est doux comme une couverture. On va voir le pain, papa ? Oui. On va marcher jusqu'à la vitrine. Papa prend les clés. Sarah avance vers la porte. Papa tend le manteau jaune. Une manche est un peu tordue. Le bras de Sarah ne glisse pas. Ça coince. Attends. Je tiens la manche ouverte. Sarah enfile une manche. Puis l'autre manche. Le tissu est doux sur ses bras. Tu veux le foulard aussi ? Oui. Il est rayé. Papa noue le foulard tout doux. On peut sortir. Papa ouvre la porte. L'air de la rue est frais. Ça sent le pain chaud. Ils marchent près. Sarah tient la main de papa. J'ai chaud dans le manteau. Oui. Parce que tu l'as pris. Ils marchent encore un peu. Un pigeon picore près du trottoir. Tu as vu le pigeon ? Oui. Il picore. Une vitrine brille. Le pain est derrière la vitre. Tu as vu le pain ? Il est doré. On le regarde un moment ? Oui. Sarah pose le front près de la vitre. La vitre est un peu froide. Le pain brille comme le soleil. C'est l'heure de rentrer. Ils rentrent. Le hall est calme. Sarah retire le manteau jaune. Elle le raccroche au crochet. Le crochet fait un petit bruit. Elle pose le foulard sur la rampe. Tu as fini de poser le foulard ? Oui. Sur la rampe. Le manteau est au crochet. Oui. Tu as su.</t>
+          <t>Un filet d'air passe sous la porte du hall. Il sent le pain chaud, venu de la rue. Sarah connaît ce hall. Les crochets, la rampe, le clou des clés. Sur le clou, un éclat de clé brille. Les clés tintent, légères. Il brille, papa. Sarah, tu as vu l'éclat ? Oui, sur la petite clé. Le manteau jaune attend au crochet. Le tissu est épais, un peu rêche. Un foulard rayé dort sur la rampe. Il est bleu et blanc. Le carrelage du hall est froid. Sarah, tu sens le pain ? Oui, papa. Je le veux à la vitrine, maintenant ! La vitrine est au bout de la rue. On y va ! On prend le manteau, d'abord. En ce moment, Sarah saisit le manteau jaune. Elle le tire d'un coup, trop vite. Une manche est tordue, à l'envers. Le bras de Sarah ne glisse pas. Ça coince ! Elle tire plus fort. La manche refuse. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Les clés de papa pendent à un clou. Elles font une petite chanson. Un foulard dort sur la rampe. Il est rayé, bleu et blanc. Sous la porte, un filet d'air froid. La rue sent déjà le pain. Sarah, tu as entendu les clés ? Oui, papa. Elles tintent. En ce moment, Sarah écoute les clés. Son manteau jaune attend au crochet. Le tissu est doux comme une couverture. On va voir le pain, papa ? Oui. On va marcher jusqu'à la vitrine. Papa prend les clés. Sarah avance vers la porte. Papa tend le manteau jaune. Une manche est un peu tordue. Le bras de Sarah ne glisse pas. Ça coince. Attends. Je tiens la manche ouverte. Sarah enfile une manche. Puis l'autre manche. Le tissu est doux sur ses bras. Tu veux le foulard aussi ? Oui. Il est rayé. Papa noue le foulard tout doux. On peut sortir. Papa ouvre la porte. L'air de la rue est frais. Ça sent le pain chaud. Ils marchent près. Sarah tient la main de papa. J'ai chaud dans le manteau. Oui. Parce que tu l'as pris. Ils marchent encore un peu. Un pigeon picore près du trottoir. Tu as vu le pigeon ? Oui. Il picore. Une vitrine brille. Le pain est derrière la vitre. Tu as vu le pain ? Il est doré. On le regarde un moment ? Oui. Sarah pose le front près de la vitre. La vitre est un peu froide. Le pain brille comme le soleil. C'est l'heure de rentrer. Ils rentrent. Le hall est calme. Sarah retire le manteau jaune. Elle le raccroche au crochet. Le crochet fait un petit bruit. Elle pose le foulard sur la rampe. Tu as fini de poser le foulard ? Oui. Sur la rampe. Le manteau est au crochet. Oui. Tu as su.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un filet d'air passe sous la porte du hall. Il sent le pain chaud, venu de la rue. Sarah connaît ce hall. Les crochets, la rampe, le clou des clés. Sur le clou, un &lt;emphasis level="moderate"&gt;éclat de clé&lt;/emphasis&gt; brille. Les clés tintent, légères. Il brille, papa. Sarah, tu as vu l'éclat ? Oui, sur la petite clé. Le manteau jaune attend au crochet. Le tissu est épais, un peu rêche. Un foulard rayé dort sur la rampe. Il est bleu et blanc. Le carrelage du hall est froid. Sarah, tu sens le pain ? Oui, papa. Je le veux à la vitrine, maintenant ! La vitrine est au bout de la rue. On y va ! On prend le manteau, d'abord. En ce moment, Sarah saisit le manteau jaune. Elle le tire d'un coup, trop vite. Une manche est tordue, à l'envers. Le bras de Sarah ne glisse pas. Ça coince ! Elle tire plus fort. La manche refuse. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Sara veut sortir avec papa. Ils sont dans le hall. L'air de la porte est frais. Papa prend le &lt;emphasis&gt;manteau&lt;/emphasis&gt;. Sara enfile le manteau. Le tissu est doux. Ils sortent. La rue sent le pain. Parce qu'elle a le manteau, Sara a chaud. Ils marchent près. Puis ils rentrent. Sara retire le manteau. Elle le pose à sa place. Elle le raccroche. Le crochet fait un petit bruit. Papa dit : manteau pour sortir. Manteau à sa place en rentrant. Sara hoche la tête. Elle a su prendre le manteau. Elle a su le raccrocher. [pause]</t>
+          <t>Un filet d'air passe sous la porte du hall. Il sent le pain chaud, venu de la rue. Sarah connaît ce hall. Les crochets, la rampe, le clou des clés. Sur le clou, un &lt;emphasis&gt;éclat de clé&lt;/emphasis&gt; brille. Les clés tintent, légères. Il brille, papa. Sarah, tu as vu l'éclat ? Oui, sur la petite clé. Le manteau jaune attend au crochet. Le tissu est épais, un peu rêche. Un foulard rayé dort sur la rampe. Il est bleu et blanc. Le carrelage du hall est froid. Sarah, tu sens le pain ? Oui, papa. Je le veux à la vitrine, maintenant ! La vitrine est au bout de la rue. On y va ! On prend le manteau, d'abord. En ce moment, Sarah saisit le manteau jaune. Elle le tire d'un coup, trop vite. Une manche est tordue, à l'envers. Le bras de Sarah ne glisse pas. Ça coince ! Elle tire plus fort. La manche refuse. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>manteau</t>
+          <t>éclat de clé</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,75 +1321,42 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_pain_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Les clés de papa pendent à un clou.
-narrateur|Elles font une petite chanson.
-narrateur|Un foulard dort sur la rampe.
-narrateur|Il est rayé, bleu et blanc.
-narrateur|Sous la porte, un filet d'air froid.
-narrateur|La rue sent déjà le pain.
-papa|Sarah, tu as entendu les clés ?
+          <t>narrateur|Un filet d'air passe sous la porte du hall.
+narrateur|Il sent le pain chaud, venu de la rue.
+narrateur|Sarah connaît ce hall.
+narrateur|Les crochets, la rampe, le clou des clés.
+narrateur|Sur le clou, un éclat de clé brille.
+narrateur|Les clés tintent, légères.
+enfant-f|Il brille, papa.
+papa|Sarah, tu as vu l'éclat ?
+enfant-f|Oui, sur la petite clé.
+narrateur|Le manteau jaune attend au crochet.
+narrateur|Le tissu est épais, un peu rêche.
+narrateur|Un foulard rayé dort sur la rampe.
+narrateur|Il est bleu et blanc.
+narrateur|Le carrelage du hall est froid.
+papa|Sarah, tu sens le pain ?
 enfant-f|Oui, papa.
-enfant-f|Elles tintent.
-narrateur|En ce moment, Sarah écoute les clés.
-narrateur|Son manteau jaune attend au crochet.
-narrateur|Le tissu est doux comme une couverture.
-enfant-f|On va voir le pain, papa ?
-papa|Oui.
-papa|On va marcher jusqu'à la vitrine.
-narrateur|Papa prend les clés.
-narrateur|Sarah avance vers la porte.
-narrateur|Papa tend le manteau jaune.
-narrateur|Une manche est un peu tordue.
+enfant-f|Je le veux à la vitrine, maintenant !
+papa|La vitrine est au bout de la rue.
+enfant-f|On y va !
+papa|On prend le manteau, d'abord.
+narrateur|En ce moment, Sarah saisit le manteau jaune.
+narrateur|Elle le tire d'un coup, trop vite.
+narrateur|Une manche est tordue, à l'envers.
 narrateur|Le bras de Sarah ne glisse pas.
-enfant-f|Ça coince.
-papa|Attends.
-papa|Je tiens la manche ouverte.
-narrateur|Sarah enfile une manche.
-narrateur|Puis l'autre manche.
-narrateur|Le tissu est doux sur ses bras.
-papa|Tu veux le foulard aussi ?
-enfant-f|Oui.
-enfant-f|Il est rayé.
-narrateur|Papa noue le foulard tout doux.
-papa|On peut sortir.
-narrateur|Papa ouvre la porte.
-narrateur|L'air de la rue est frais.
-narrateur|Ça sent le pain chaud.
-narrateur|Ils marchent près.
-narrateur|Sarah tient la main de papa.
-enfant-f|J'ai chaud dans le manteau.
-papa|Oui.
-papa|Parce que tu l'as pris.
-narrateur|Ils marchent encore un peu.
-narrateur|Un pigeon picore près du trottoir.
-papa|Tu as vu le pigeon ?
-enfant-f|Oui.
-enfant-f|Il picore.
-narrateur|Une vitrine brille.
-narrateur|Le pain est derrière la vitre.
-papa|Tu as vu le pain ?
-enfant-f|Il est doré.
-papa|On le regarde un moment ?
-enfant-f|Oui.
-narrateur|Sarah pose le front près de la vitre.
-narrateur|La vitre est un peu froide.
-narrateur|Le pain brille comme le soleil.
-papa|C'est l'heure de rentrer.
-narrateur|Ils rentrent.
-narrateur|Le hall est calme.
-narrateur|Sarah retire le manteau jaune.
-narrateur|Elle le raccroche au crochet.
-narrateur|Le crochet fait un petit bruit.
-narrateur|Elle pose le foulard sur la rampe.
-papa|Tu as fini de poser le foulard ?
-enfant-f|Oui.
-enfant-f|Sur la rampe.
-enfant-f|Le manteau est au crochet.
-papa|Oui.
-papa|Tu as su.</t>
+enfant-f|Ça coince !
+narrateur|Elle tire plus fort.
+narrateur|La manche refuse.
+narrateur|Le sourire de Sarah disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1426,12 +1393,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Sarah va dehors. Que prend-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah va &lt;emphasis level="moderate"&gt;dehors&lt;/emphasis&gt;. Que prend-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Sara va dehors. Que prend-el&lt;emphasis&gt;le&lt;/emphasis&gt; ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Sarah va &lt;emphasis&gt;dehors&lt;/emphasis&gt;. Que prend-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1441,7 +1408,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>le manteau | manteau | elle l'enfile</t>
+          <t>le manteau | manteau | elle l'enfile | le manteau jaune</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1494,7 +1461,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1505,7 +1472,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.22</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1520,38 +1487,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
-          <t>le</t>
+          <t>dehors</t>
         </is>
       </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1566,17 +1533,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_prend_le_manteau; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1609,17 +1576,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sarah a pris le manteau jaune. Elle l'a mis pour la rue. Elle a vu le pain doré. En rentrant, elle a raccroché. Tu as pris le manteau pour sortir. Il est à sa place. Oui. Avec le foulard sur la rampe.</t>
+          <t>Papa s'accroupit à la même hauteur. Tu regardes la manche ? Je veux le pain, papa. Sarah refuse de tirer plus fort. Elle pose un genou au sol. La manche est plate, à l'envers. Je la tourne. Elle retourne le tissu, sans forcer. Le bras glisse, petit à petit. Elle est ouverte. Merci, Sarah. Elle enfile l'autre manche. Le tissu est chaud sur ses bras. Tu veux le foulard aussi ? Oui, il est rayé. Papa noue le foulard, près du cou. On ouvre la porte ? Oui, papa. Papa ouvre la porte du hall. L'air de la rue est frais. Ça sent le pain chaud. Sarah tient la main de papa. J'ai chaud dans le manteau. Oui, parce que tu l'as pris.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sarah a pris le manteau jaune. Elle l'a mis pour la rue. Elle a vu le pain doré. En rentrant, elle a raccroché. Tu as pris le manteau pour sortir. Il est à sa place. Oui. Avec le foulard sur la rampe.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Papa s'accroupit à la même hauteur. Tu regardes la &lt;emphasis level="moderate"&gt;manche&lt;/emphasis&gt; ? Je veux le pain, papa. Sarah refuse de tirer plus fort. Elle pose un genou au sol. La manche est plate, à l'envers. Je la tourne. Elle retourne le tissu, sans forcer. Le bras glisse, petit à petit. Elle est ouverte. Merci, Sarah. Elle enfile l'autre manche. Le tissu est chaud sur ses bras. Tu veux le foulard aussi ? Oui, il est rayé. Papa noue le foulard, près du cou. On ouvre la porte ? Oui, papa. Papa ouvre la porte du hall. L'air de la rue est frais. Ça sent le pain chaud. Sarah tient la main de papa. J'ai chaud dans le manteau. Oui, parce que tu l'as pris.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Sara a pris le &lt;emphasis&gt;manteau&lt;/emphasis&gt; pour sortir. En rentrant, elle l'a raccroché. Papa était là. [pause]</t>
+          <t>Papa s'accroupit à la même hauteur. Tu regardes la &lt;emphasis&gt;manche&lt;/emphasis&gt; ? Je veux le pain, papa. Sarah refuse de tirer plus fort. Elle pose un genou au sol. La manche est plate, à l'envers. Je la tourne. Elle retourne le tissu, sans forcer. Le bras glisse, petit à petit. Elle est ouverte. Merci, Sarah. Elle enfile l'autre manche. Le tissu est chaud sur ses bras. Tu veux le foulard aussi ? Oui, il est rayé. Papa noue le foulard, près du cou. On ouvre la porte ? Oui, papa. Papa ouvre la porte du hall. L'air de la rue est frais. Ça sent le pain chaud. Sarah tient la main de papa. J'ai chaud dans le manteau. Oui, parce que tu l'as pris. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1677,7 +1644,7 @@
         <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1700,7 +1667,7 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>manteau</t>
+          <t>manche</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
@@ -1714,16 +1681,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1748,19 +1715,40 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=1; destinataire=enfant; sous_texte=elle_ouvre_la_manche_sans_forcer; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Sarah a pris le manteau jaune.
-narrateur|Elle l'a mis pour la rue.
-narrateur|Elle a vu le pain doré.
-narrateur|En rentrant, elle a raccroché.
-papa|Tu as pris le manteau pour sortir.
-enfant-f|Il est à sa place.
-papa|Oui.
-papa|Avec le foulard sur la rampe.</t>
+          <t>narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu regardes la manche ?
+enfant-f|Je veux le pain, papa.
+narrateur|Sarah refuse de tirer plus fort.
+narrateur|Elle pose un genou au sol.
+narrateur|La manche est plate, à l'envers.
+enfant-f|Je la tourne.
+narrateur|Elle retourne le tissu, sans forcer.
+narrateur|Le bras glisse, petit à petit.
+enfant-f|Elle est ouverte.
+papa|Merci, Sarah.
+narrateur|Elle enfile l'autre manche.
+narrateur|Le tissu est chaud sur ses bras.
+papa|Tu veux le foulard aussi ?
+enfant-f|Oui, il est rayé.
+narrateur|Papa noue le foulard, près du cou.
+papa|On ouvre la porte ?
+enfant-f|Oui, papa.
+narrateur|Papa ouvre la porte du hall.
+narrateur|L'air de la rue est frais.
+narrateur|Ça sent le pain chaud.
+narrateur|Sarah tient la main de papa.
+enfant-f|J'ai chaud dans le manteau.
+papa|Oui, parce que tu l'as pris.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>manteau,foulard</t>
         </is>
       </c>
     </row>
@@ -1787,17 +1775,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose ses chaussures. Elles restent près du paillasson. Tu as fini de poser tes chaussures ? Oui, papa. Papa ferme la porte. Le filet d'air s'arrête. Les clés redeviennent silencieuses. On reste au chaud, maintenant. Le pain était doré. Oui. Et le manteau attend au crochet.</t>
+          <t>Ils marchent près, sur le trottoir. Le manteau jaune tape contre sa hanche. Je le vois, papa ? Bientôt. Une enseigne claque, plus loin. Le trottoir sent la farine. Je cours jusqu'à la vitrine ! Sarah veut glisser entre un cageot et le mur. Le cageot de sacs bloque le passage. Elle pousse, d'un coup. La manche jaune s'accroche à une latte. Ça tient ! Elle tire. Le cageot penche un peu. Sarah s'arrête net. Je n'aime pas ça. Elle refuse de foncer. Attends, je regarde. Papa ne parle pas. Sarah observe les clés, puis le cageot. Dans la main de papa, les clés tintent. L'éclat de clé brille dans un trou, à droite. Par là, papa. Tu vois le trou ? Oui, l'éclat le montre. Ils contournent le cageot, sans se presser. La vitrine est libre. Le pain doré attend derrière le verre. Il est là. Oui, il est près.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sarah pose ses chaussures. Elles restent près du paillasson. Tu as fini de poser tes chaussures ? Oui, papa. Papa ferme la porte. Le filet d'air s'arrête. Les clés redeviennent silencieuses. On reste au chaud, maintenant. Le pain était doré. Oui. Et le manteau attend au crochet.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils marchent près, sur le trottoir. Le manteau jaune tape contre sa hanche. Je le vois, papa ? Bientôt. Une enseigne claque, plus loin. Le trottoir sent la farine. Je cours jusqu'à la vitrine ! Sarah veut glisser entre un cageot et le mur. Le cageot de sacs bloque le passage. Elle pousse, d'un coup. La manche jaune s'accroche à une latte. Ça tient ! Elle tire. Le cageot penche un peu. Sarah s'arrête net. Je n'aime pas ça. Elle refuse de foncer. Attends, je regarde. Papa ne parle pas. Sarah observe les clés, puis le cageot. Dans la main de papa, les clés tintent. L'&lt;emphasis level="moderate"&gt;éclat de clé&lt;/emphasis&gt; brille dans un trou, à droite. Par là, papa. Tu vois le trou ? Oui, l'éclat le montre. Ils contournent le cageot, sans se presser. La vitrine est libre. Le pain doré attend derrière le verre. Il est là. Oui, il est près.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Sara pose ses chaussures. Papa ferme la porte. [pause]</t>
+          <t>Ils marchent près, sur le trottoir. Le manteau jaune tape contre sa hanche. Je le vois, papa ? Bientôt. Une enseigne claque, plus loin. Le trottoir sent la farine. Je cours jusqu'à la vitrine ! Sarah veut glisser entre un cageot et le mur. Le cageot de sacs bloque le passage. Elle pousse, d'un coup. La manche jaune s'accroche à une latte. Ça tient ! Elle tire. Le cageot penche un peu. Sarah s'arrête net. Je n'aime pas ça. Elle refuse de foncer. Attends, je regarde. Papa ne parle pas. Sarah observe les clés, puis le cageot. Dans la main de papa, les clés tintent. L'&lt;emphasis&gt;éclat de clé&lt;/emphasis&gt; brille dans un trou, à droite. Par là, papa. Tu vois le trou ? Oui, l'éclat le montre. Ils contournent le cageot, sans se presser. La vitrine est libre. Le pain doré attend derrière le verre. Il est là. Oui, il est près. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1844,7 +1832,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1852,10 +1840,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1876,28 +1864,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de clé</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1906,10 +1898,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1920,20 +1912,48 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=résolution; intention=faire_vivre_la_réussite; emotion=élan puis prudence puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_l_éclat_montre_le_trou; tempo=vif puis posé; sourire=léger; respiration=relâchée</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Sarah pose ses chaussures.
-narrateur|Elles restent près du paillasson.
-papa|Tu as fini de poser tes chaussures ?
-enfant-f|Oui, papa.
-narrateur|Papa ferme la porte.
-narrateur|Le filet d'air s'arrête.
-narrateur|Les clés redeviennent silencieuses.
-papa|On reste au chaud, maintenant.
-enfant-f|Le pain était doré.
-papa|Oui.
-papa|Et le manteau attend au crochet.</t>
+          <t>narrateur|Ils marchent près, sur le trottoir.
+narrateur|Le manteau jaune tape contre sa hanche.
+enfant-f|Je le vois, papa ?
+papa|Bientôt.
+narrateur|Une enseigne claque, plus loin.
+narrateur|Le trottoir sent la farine.
+enfant-f|Je cours jusqu'à la vitrine !
+narrateur|Sarah veut glisser entre un cageot et le mur.
+narrateur|Le cageot de sacs bloque le passage.
+narrateur|Elle pousse, d'un coup.
+narrateur|La manche jaune s'accroche à une latte.
+enfant-f|Ça tient !
+narrateur|Elle tire.
+narrateur|Le cageot penche un peu.
+narrateur|Sarah s'arrête net.
+enfant-f|Je n'aime pas ça.
+narrateur|Elle refuse de foncer.
+enfant-f|Attends, je regarde.
+narrateur|Papa ne parle pas.
+narrateur|Sarah observe les clés, puis le cageot.
+narrateur|Dans la main de papa, les clés tintent.
+narrateur|L'éclat de clé brille dans un trou, à droite.
+enfant-f|Par là, papa.
+papa|Tu vois le trou ?
+enfant-f|Oui, l'éclat le montre.
+narrateur|Ils contournent le cageot, sans se presser.
+narrateur|La vitrine est libre.
+narrateur|Le pain doré attend derrière le verre.
+enfant-f|Il est là.
+papa|Oui, il est près.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>rue,pas</t>
         </is>
       </c>
     </row>
@@ -1960,17 +1980,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai vu le pain doré. J'avais le manteau pour la rue. Bravo, Sarah. Le pain sent encore sous la porte.</t>
+          <t>Sarah pose le front près de la vitre. La vitre est un peu froide. Le pain est doré. Oui, il est chaud. Papa tient les clés contre le verre. Sur la croûte, un éclat de clé brille. Comme sur le clou, papa ! Tu le vois, toi ? Oui, il est sur le pain. Ils rentrent vers le hall. Sarah retire le manteau jaune. Elle le raccroche au crochet. Le crochet fait un petit bruit. Elle pose le foulard sur la rampe. Tu as fini de poser le foulard ? Oui, sur la rampe. Les clés retrouvent le clou. Le pain sent sous la porte.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai vu le pain doré. J'avais le manteau pour la rue. Bravo, Sarah. Le pain sent encore sous la porte.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sarah pose le front près de la vitre. La vitre est un peu froide. Le pain est doré. Oui, il est chaud. Papa tient les clés contre le verre. Sur la croûte, un &lt;emphasis level="moderate"&gt;éclat de clé&lt;/emphasis&gt; brille. Comme sur le clou, papa ! Tu le vois, toi ? Oui, il est sur le pain. Ils rentrent vers le hall. Sarah retire le manteau jaune. Elle le raccroche au crochet. Le crochet fait un petit bruit. Elle pose le foulard sur la rampe. Tu as fini de poser le foulard ? Oui, sur la rampe. Les clés retrouvent le clou. Le pain sent sous la porte.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sarah pose le front près de la vitre. La vitre est un peu froide. Le pain est doré. Oui, il est chaud. Papa tient les clés contre le verre. Sur la croûte, un &lt;emphasis&gt;éclat de clé&lt;/emphasis&gt; brille. Comme sur le clou, papa ! Tu le vois, toi ? Oui, il est sur le pain. Ils rentrent vers le hall. Sarah retire le manteau jaune. Elle le raccroche au crochet. Le crochet fait un petit bruit. Elle pose le foulard sur la rampe. Tu as fini de poser le foulard ? Oui, sur la rampe. Les clés retrouvent le clou. Le pain sent sous la porte.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2017,7 +2037,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2025,7 +2045,7 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2037,12 +2057,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2051,17 +2071,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de clé</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2070,11 +2094,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2083,27 +2107,50 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_éclat_du_clou_est_sur_la_croute; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai vu le pain doré.
-enfant-f|J'avais le manteau pour la rue.
-papa|Bravo, Sarah.
-narrateur|Le pain sent encore sous la porte.</t>
+          <t>narrateur|Sarah pose le front près de la vitre.
+narrateur|La vitre est un peu froide.
+enfant-f|Le pain est doré.
+papa|Oui, il est chaud.
+narrateur|Papa tient les clés contre le verre.
+narrateur|Sur la croûte, un éclat de clé brille.
+enfant-f|Comme sur le clou, papa !
+papa|Tu le vois, toi ?
+enfant-f|Oui, il est sur le pain.
+narrateur|Ils rentrent vers le hall.
+narrateur|Sarah retire le manteau jaune.
+narrateur|Elle le raccroche au crochet.
+narrateur|Le crochet fait un petit bruit.
+narrateur|Elle pose le foulard sur la rampe.
+papa|Tu as fini de poser le foulard ?
+enfant-f|Oui, sur la rampe.
+narrateur|Les clés retrouvent le clou.
+narrateur|Le pain sent sous la porte.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>vitrine,cles</t>
         </is>
       </c>
     </row>
@@ -2124,7 +2171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2216,6 +2263,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>